<commit_message>
commit truoc khi chuyen nhanh
</commit_message>
<xml_diff>
--- a/templates/template_tasks.xlsx
+++ b/templates/template_tasks.xlsx
@@ -611,24 +611,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P957"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
-    <col min="13" max="13" width="20.83203125" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" customWidth="1"/>
-    <col min="15" max="15" width="20.83203125" customWidth="1"/>
-    <col min="16" max="16" width="30.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -972,20 +954,18 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1000"/>
+  <dimension ref="A1:B3"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Owners</v>
       </c>
       <c r="B1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Priority</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Phase</v>
+        <v>Name</v>
       </c>
     </row>
     <row r="2">
@@ -993,13 +973,7 @@
         <v>BE 1</v>
       </c>
       <c r="B2" t="str">
-        <v>To Do</v>
-      </c>
-      <c r="C2" t="str">
-        <v>P0</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Phase 1 - Foundation</v>
+        <v>Nguyễn Văn A</v>
       </c>
     </row>
     <row r="3">
@@ -1007,46 +981,12 @@
         <v>BE 2</v>
       </c>
       <c r="B3" t="str">
-        <v>In Progress</v>
-      </c>
-      <c r="C3" t="str">
-        <v>P1</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Phase 2 - API Core</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>BE 3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Review</v>
-      </c>
-      <c r="C4" t="str">
-        <v>P2</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Phase 3 - Enhancement</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" t="str">
-        <v>Done</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Phase 4 - Stabilization</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="str">
-        <v>Blocked</v>
+        <v>Trần Thị B</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M1000"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>